<commit_message>
Update scaffold with renewed ChemLib 7.21 xlsx
- Fix E266 SMILES (chemically impossible valence → trifluoromethoxy)
- Regenerate JSON/YAML and all 895 scaffold SVGs
- H018/H021 still use CD3→CH3 fallback; J128/J129 use unsanitized fallback
</commit_message>
<xml_diff>
--- a/_chemlib_data/scaffold_ZhangLab_ChemLib_7.21.xlsx
+++ b/_chemlib_data/scaffold_ZhangLab_ChemLib_7.21.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="10680" windowHeight="11610"/>
+    <workbookView windowWidth="28800" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4985,7 +4985,7 @@
     <t>E266</t>
   </si>
   <si>
-    <t>O=C(NCC(C=C1)=CC2=C1C(N(C2)C(C(N3)=O)CCC3=O)=O)C(C4=CNC5=C4C=C(C(F)(F)(F)=O)C=C5)C6=CC=CC=C6</t>
+    <t>O=C(NCC(C=C1)=CC2=C1C(N(C2)C(C(N3)=O)CCC3=O)=O)C(C4=CNC5=C4C=C(OC(F)(F)F)C=C5)C6=CC=CC=C6</t>
   </si>
   <si>
     <t>ZR-583</t>

</xml_diff>